<commit_message>
feat: add Daily Sadhana.xlsx to public directory
</commit_message>
<xml_diff>
--- a/public/Daily Sadhana.xlsx
+++ b/public/Daily Sadhana.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sahaa\Documents\github_anandasvarupa\give_web\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8816264A-140B-4C26-9259-258AA92B200F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F38CE409-430D-413E-981A-618BE0ABA058}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BS-4" sheetId="1" r:id="rId1"/>
     <sheet name="BS-5" sheetId="2" r:id="rId2"/>
     <sheet name="BS-Ekacakra" sheetId="3" r:id="rId3"/>
+    <sheet name="BS-2-English" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1273" uniqueCount="528">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1308" uniqueCount="544">
   <si>
     <t>url</t>
   </si>
@@ -1612,6 +1613,54 @@
   <si>
     <t>Today's listening to Srila Prabhupada - 289</t>
   </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1120</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1121</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1122</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1123</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1124</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1125</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1126</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1127</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1128</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1129</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1130</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1131</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1132</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1133</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1134</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1135</t>
+  </si>
 </sst>
 </file>
 
@@ -1621,7 +1670,7 @@
     <numFmt numFmtId="164" formatCode="mmm\ d\,\ yy"/>
     <numFmt numFmtId="165" formatCode="mmm\ d\,\ yyyy"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -1658,6 +1707,11 @@
       <sz val="8"/>
       <name val="Arial"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Arial"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -60549,4 +60603,249 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2DB8064-9FCF-4672-A5DD-AAA1AF5AE7B8}">
+  <dimension ref="A1:Z17"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="50.90625" customWidth="1"/>
+    <col min="2" max="2" width="38.90625" customWidth="1"/>
+    <col min="3" max="3" width="28.90625" customWidth="1"/>
+    <col min="4" max="4" width="21.36328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+      <c r="M1" s="2"/>
+      <c r="N1" s="2"/>
+      <c r="O1" s="2"/>
+      <c r="P1" s="2"/>
+      <c r="Q1" s="2"/>
+      <c r="R1" s="2"/>
+      <c r="S1" s="2"/>
+      <c r="T1" s="2"/>
+      <c r="U1" s="2"/>
+      <c r="V1" s="2"/>
+      <c r="W1" s="2"/>
+      <c r="X1" s="2"/>
+      <c r="Y1" s="2"/>
+      <c r="Z1" s="2"/>
+    </row>
+    <row r="2" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="11" t="s">
+        <v>446</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>528</v>
+      </c>
+      <c r="C2" s="7">
+        <v>46280</v>
+      </c>
+    </row>
+    <row r="3" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="11" t="s">
+        <v>447</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>529</v>
+      </c>
+      <c r="C3" s="7">
+        <v>46281</v>
+      </c>
+    </row>
+    <row r="4" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="11" t="s">
+        <v>448</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>530</v>
+      </c>
+      <c r="C4" s="7">
+        <v>46282</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="11" t="s">
+        <v>449</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>531</v>
+      </c>
+      <c r="C5" s="7">
+        <v>46283</v>
+      </c>
+    </row>
+    <row r="6" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="11" t="s">
+        <v>450</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>532</v>
+      </c>
+      <c r="C6" s="7">
+        <v>46284</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="11" t="s">
+        <v>451</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>533</v>
+      </c>
+      <c r="C7" s="7">
+        <v>46285</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="11" t="s">
+        <v>452</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>534</v>
+      </c>
+      <c r="C8" s="7">
+        <v>46286</v>
+      </c>
+    </row>
+    <row r="9" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="11" t="s">
+        <v>453</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>535</v>
+      </c>
+      <c r="C9" s="7">
+        <v>46287</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="11" t="s">
+        <v>454</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>536</v>
+      </c>
+      <c r="C10" s="7">
+        <v>46288</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="11" t="s">
+        <v>455</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>537</v>
+      </c>
+      <c r="C11" s="7">
+        <v>46289</v>
+      </c>
+    </row>
+    <row r="12" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="11" t="s">
+        <v>456</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>538</v>
+      </c>
+      <c r="C12" s="7">
+        <v>46290</v>
+      </c>
+    </row>
+    <row r="13" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="11" t="s">
+        <v>457</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>539</v>
+      </c>
+      <c r="C13" s="7">
+        <v>46291</v>
+      </c>
+    </row>
+    <row r="14" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="11" t="s">
+        <v>458</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>540</v>
+      </c>
+      <c r="C14" s="7">
+        <v>46292</v>
+      </c>
+    </row>
+    <row r="15" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="11" t="s">
+        <v>459</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>541</v>
+      </c>
+      <c r="C15" s="7">
+        <v>46293</v>
+      </c>
+    </row>
+    <row r="16" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="11" t="s">
+        <v>460</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>542</v>
+      </c>
+      <c r="C16" s="7">
+        <v>46294</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="11" t="s">
+        <v>312</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>543</v>
+      </c>
+      <c r="C17" s="7">
+        <v>46295</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="6" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1" display="https://www.youtube.com/watch?v=1Ilgi75Y6Ac&amp;t=9s" xr:uid="{BEFFE2FC-FF84-4042-B8EC-77144312CABC}"/>
+    <hyperlink ref="A3" r:id="rId2" xr:uid="{90F813C6-4FEA-4DED-83BD-5034A555CC22}"/>
+    <hyperlink ref="A4" r:id="rId3" xr:uid="{B1C314CD-370C-4CA6-9FE8-1ED3943E31D4}"/>
+    <hyperlink ref="A5" r:id="rId4" xr:uid="{A17D0F69-B2D0-46D9-B6F6-66C068704A56}"/>
+    <hyperlink ref="A6" r:id="rId5" display="https://www.youtube.com/watch?v=zgLWXkOMOGE&amp;t=20s" xr:uid="{9779AA05-4C44-47F0-B170-2FE8FB47B3BE}"/>
+    <hyperlink ref="A7" r:id="rId6" display="https://www.youtube.com/watch?v=r-DPvpwMOdw&amp;t=144s" xr:uid="{0276A8C9-E8B0-4D6A-9CEF-9F2AAB75C880}"/>
+    <hyperlink ref="A8" r:id="rId7" xr:uid="{F19BACE9-B34B-4C91-86EB-670079642404}"/>
+    <hyperlink ref="A9" r:id="rId8" xr:uid="{7CBC5B68-7623-491F-8129-5C469970DB0C}"/>
+    <hyperlink ref="A10" r:id="rId9" xr:uid="{6503D671-ACE1-4397-8206-9F396EA2AA88}"/>
+    <hyperlink ref="A11" r:id="rId10" xr:uid="{3DAB877A-772C-41D4-9E5C-E44AFD14063A}"/>
+    <hyperlink ref="A12" r:id="rId11" display="https://www.youtube.com/watch?v=X6XNEMBmPrk&amp;t=149s" xr:uid="{3D449635-2546-48EE-9157-EDAADD1D323B}"/>
+    <hyperlink ref="A13" r:id="rId12" xr:uid="{ADF479E2-4D26-4E3A-8975-974F3667CD5A}"/>
+    <hyperlink ref="A14" r:id="rId13" xr:uid="{DE18D8BB-EB17-4E0B-B273-35819EBED68A}"/>
+    <hyperlink ref="A15" r:id="rId14" display="https://www.youtube.com/watch?v=qCOWcKURVzk&amp;t=1s" xr:uid="{6A11C7B1-0010-43D5-9F17-1F6D51AD59E6}"/>
+    <hyperlink ref="A16" r:id="rId15" xr:uid="{AD44B6A8-1E3C-44E6-A013-F6004413BDEA}"/>
+    <hyperlink ref="A17" r:id="rId16" display="https://www.youtube.com/watch?v=-NHHdVWUcwo&amp;t=3s" xr:uid="{B9FC0606-31ED-4E7D-91D6-1FC640AB21A4}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
NOD Listening added to BS#2 English
</commit_message>
<xml_diff>
--- a/public/Daily Sadhana.xlsx
+++ b/public/Daily Sadhana.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sahaa\Documents\github_anandasvarupa\give_web\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F38CE409-430D-413E-981A-618BE0ABA058}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD15EB56-47F7-4302-A672-84AE5291562B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5170" yWindow="3470" windowWidth="14030" windowHeight="6610" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BS-4" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1308" uniqueCount="544">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1362" uniqueCount="611">
   <si>
     <t>url</t>
   </si>
@@ -1661,6 +1661,207 @@
   <si>
     <t>Today's listening to Srila Prabhupada - 1135</t>
   </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=CftLOpEg8JM</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=zsCVrqVMcx8</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=ECzOXYCimqs</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=YLO02uvW1jw</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=zsTa0XXJ7qo</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=CWoOXeF3Yxg</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=bE_ippUqgo0</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=AwMpoLPpteI</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=US55Ai355ag</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=yPoaMCjJln4</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=4x6esIcwhK0</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=j7T1MKt-ydA</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=CL3MjqFWpRk</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=EtaDH-J1ZEY</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=STe9eE9d6cM</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=bXGdE7t5DHg</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=1LDGcLBVSuk</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=GvZbTG9Hwj8</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=zhOO4Svlg0g</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=Tw3vp5zupx0</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=KX4XKIQ558I</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=5IdV68D4A90</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=aN2y6k1zMa4</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=PSEXwM2qQmM</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=8siMw00cRt8</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=6S_PSfha1ag</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=bYF_FX-vZ78</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=f8AoUoiTXes</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=iUJA3Bh8NzE</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=GiMnzOTvMOM</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=ixeML2iYD3w</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=H9h2FMQPUeg</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=yi3n-KpYdVY</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=GDeMHEPvhIw</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=tp3q1RMK2cw</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=VTg-IZm0q34</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=OaIUX41Sz48</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=VcS7IKB-d8s</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=3iX21gh2t0Q</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=yiug7xQlTAI</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1136</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1137</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1138</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1139</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1140</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1141</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1142</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1143</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1144</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1145</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1146</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1147</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1148</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1149</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1150</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1151</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1152</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1153</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1154</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1155</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1156</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1157</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1158</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1159</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1160</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1161</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1162</t>
+  </si>
 </sst>
 </file>
 
@@ -1802,7 +2003,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1843,6 +2044,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -60607,7 +60809,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2DB8064-9FCF-4672-A5DD-AAA1AF5AE7B8}">
-  <dimension ref="A1:Z17"/>
+  <dimension ref="A1:Z44"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="50.90625" customWidth="1"/>
@@ -60663,7 +60865,7 @@
     </row>
     <row r="3" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="11" t="s">
-        <v>447</v>
+        <v>544</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>529</v>
@@ -60674,7 +60876,7 @@
     </row>
     <row r="4" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="11" t="s">
-        <v>448</v>
+        <v>545</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>530</v>
@@ -60685,7 +60887,7 @@
     </row>
     <row r="5" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="11" t="s">
-        <v>449</v>
+        <v>546</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>531</v>
@@ -60696,7 +60898,7 @@
     </row>
     <row r="6" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
-        <v>450</v>
+        <v>547</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>532</v>
@@ -60707,7 +60909,7 @@
     </row>
     <row r="7" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
-        <v>451</v>
+        <v>548</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>533</v>
@@ -60718,7 +60920,7 @@
     </row>
     <row r="8" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
-        <v>452</v>
+        <v>549</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>534</v>
@@ -60729,7 +60931,7 @@
     </row>
     <row r="9" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
-        <v>453</v>
+        <v>550</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>535</v>
@@ -60740,7 +60942,7 @@
     </row>
     <row r="10" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="11" t="s">
-        <v>454</v>
+        <v>551</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>536</v>
@@ -60751,7 +60953,7 @@
     </row>
     <row r="11" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
-        <v>455</v>
+        <v>552</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>537</v>
@@ -60762,7 +60964,7 @@
     </row>
     <row r="12" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="11" t="s">
-        <v>456</v>
+        <v>553</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>538</v>
@@ -60773,7 +60975,7 @@
     </row>
     <row r="13" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="11" t="s">
-        <v>457</v>
+        <v>554</v>
       </c>
       <c r="B13" s="6" t="s">
         <v>539</v>
@@ -60784,7 +60986,7 @@
     </row>
     <row r="14" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
-        <v>458</v>
+        <v>555</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>540</v>
@@ -60795,7 +60997,7 @@
     </row>
     <row r="15" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="11" t="s">
-        <v>459</v>
+        <v>556</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>541</v>
@@ -60806,7 +61008,7 @@
     </row>
     <row r="16" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="11" t="s">
-        <v>460</v>
+        <v>557</v>
       </c>
       <c r="B16" s="6" t="s">
         <v>542</v>
@@ -60817,34 +61019,317 @@
     </row>
     <row r="17" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="11" t="s">
-        <v>312</v>
+        <v>558</v>
       </c>
       <c r="B17" s="6" t="s">
         <v>543</v>
       </c>
       <c r="C17" s="7">
         <v>46295</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="14" t="s">
+        <v>559</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>584</v>
+      </c>
+      <c r="C18" s="7">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>560</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>585</v>
+      </c>
+      <c r="C19" s="7">
+        <v>46297</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>561</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>586</v>
+      </c>
+      <c r="C20" s="7">
+        <v>46298</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>562</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>587</v>
+      </c>
+      <c r="C21" s="7">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>563</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>588</v>
+      </c>
+      <c r="C22" s="7">
+        <v>46300</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>564</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>589</v>
+      </c>
+      <c r="C23" s="7">
+        <v>46301</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>565</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>590</v>
+      </c>
+      <c r="C24" s="7">
+        <v>46302</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>566</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>591</v>
+      </c>
+      <c r="C25" s="7">
+        <v>46303</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>567</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>592</v>
+      </c>
+      <c r="C26" s="7">
+        <v>46304</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>568</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>593</v>
+      </c>
+      <c r="C27" s="7">
+        <v>46305</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>569</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>594</v>
+      </c>
+      <c r="C28" s="7">
+        <v>46306</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>570</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>595</v>
+      </c>
+      <c r="C29" s="7">
+        <v>46307</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>571</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>596</v>
+      </c>
+      <c r="C30" s="7">
+        <v>46308</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>572</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>597</v>
+      </c>
+      <c r="C31" s="7">
+        <v>46309</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>573</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>598</v>
+      </c>
+      <c r="C32" s="7">
+        <v>46310</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>574</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="C33" s="7">
+        <v>46311</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>422</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>600</v>
+      </c>
+      <c r="C34" s="7">
+        <v>46312</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>575</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>601</v>
+      </c>
+      <c r="C35" s="7">
+        <v>46313</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>576</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>602</v>
+      </c>
+      <c r="C36" s="7">
+        <v>46314</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>577</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>603</v>
+      </c>
+      <c r="C37" s="7">
+        <v>46315</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>578</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>604</v>
+      </c>
+      <c r="C38" s="7">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>579</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>605</v>
+      </c>
+      <c r="C39" s="7">
+        <v>46317</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>580</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>606</v>
+      </c>
+      <c r="C40" s="7">
+        <v>46318</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>581</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>607</v>
+      </c>
+      <c r="C41" s="7">
+        <v>46319</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>582</v>
+      </c>
+      <c r="B42" s="6" t="s">
+        <v>608</v>
+      </c>
+      <c r="C42" s="7">
+        <v>46320</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>366</v>
+      </c>
+      <c r="B43" s="6" t="s">
+        <v>609</v>
+      </c>
+      <c r="C43" s="7">
+        <v>46321</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>583</v>
+      </c>
+      <c r="B44" s="6" t="s">
+        <v>610</v>
+      </c>
+      <c r="C44" s="7">
+        <v>46322</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="6" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1" display="https://www.youtube.com/watch?v=1Ilgi75Y6Ac&amp;t=9s" xr:uid="{BEFFE2FC-FF84-4042-B8EC-77144312CABC}"/>
-    <hyperlink ref="A3" r:id="rId2" xr:uid="{90F813C6-4FEA-4DED-83BD-5034A555CC22}"/>
-    <hyperlink ref="A4" r:id="rId3" xr:uid="{B1C314CD-370C-4CA6-9FE8-1ED3943E31D4}"/>
-    <hyperlink ref="A5" r:id="rId4" xr:uid="{A17D0F69-B2D0-46D9-B6F6-66C068704A56}"/>
-    <hyperlink ref="A6" r:id="rId5" display="https://www.youtube.com/watch?v=zgLWXkOMOGE&amp;t=20s" xr:uid="{9779AA05-4C44-47F0-B170-2FE8FB47B3BE}"/>
-    <hyperlink ref="A7" r:id="rId6" display="https://www.youtube.com/watch?v=r-DPvpwMOdw&amp;t=144s" xr:uid="{0276A8C9-E8B0-4D6A-9CEF-9F2AAB75C880}"/>
-    <hyperlink ref="A8" r:id="rId7" xr:uid="{F19BACE9-B34B-4C91-86EB-670079642404}"/>
-    <hyperlink ref="A9" r:id="rId8" xr:uid="{7CBC5B68-7623-491F-8129-5C469970DB0C}"/>
-    <hyperlink ref="A10" r:id="rId9" xr:uid="{6503D671-ACE1-4397-8206-9F396EA2AA88}"/>
-    <hyperlink ref="A11" r:id="rId10" xr:uid="{3DAB877A-772C-41D4-9E5C-E44AFD14063A}"/>
-    <hyperlink ref="A12" r:id="rId11" display="https://www.youtube.com/watch?v=X6XNEMBmPrk&amp;t=149s" xr:uid="{3D449635-2546-48EE-9157-EDAADD1D323B}"/>
-    <hyperlink ref="A13" r:id="rId12" xr:uid="{ADF479E2-4D26-4E3A-8975-974F3667CD5A}"/>
-    <hyperlink ref="A14" r:id="rId13" xr:uid="{DE18D8BB-EB17-4E0B-B273-35819EBED68A}"/>
-    <hyperlink ref="A15" r:id="rId14" display="https://www.youtube.com/watch?v=qCOWcKURVzk&amp;t=1s" xr:uid="{6A11C7B1-0010-43D5-9F17-1F6D51AD59E6}"/>
-    <hyperlink ref="A16" r:id="rId15" xr:uid="{AD44B6A8-1E3C-44E6-A013-F6004413BDEA}"/>
-    <hyperlink ref="A17" r:id="rId16" display="https://www.youtube.com/watch?v=-NHHdVWUcwo&amp;t=3s" xr:uid="{B9FC0606-31ED-4E7D-91D6-1FC640AB21A4}"/>
+    <hyperlink ref="A18" r:id="rId2" xr:uid="{266B1484-6826-4EF7-BFC0-E28E4199D83A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: implement paginated task loading and analytics formatting improvements
</commit_message>
<xml_diff>
--- a/public/Daily Sadhana.xlsx
+++ b/public/Daily Sadhana.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sahaa\Documents\github_anandasvarupa\give_web\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{567053E3-F29A-4970-A043-06ADD0DB464C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1752A59-98D1-47C7-831C-9FBDB67F4426}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BS-4" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1728" uniqueCount="729">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1806" uniqueCount="768">
   <si>
     <t>url</t>
   </si>
@@ -2215,6 +2215,123 @@
   </si>
   <si>
     <t>Today's listening to Srila Prabhupada - 350</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1163</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1164</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1165</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1166</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1167</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1168</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1169</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1170</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1171</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1172</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1173</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1174</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1175</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1176</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1177</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1178</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1179</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1180</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1181</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1182</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1183</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1184</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1185</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1186</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1187</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1188</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1189</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1190</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1191</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1192</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1193</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1194</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1195</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1196</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1197</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1198</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1199</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1200</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 1201</t>
   </si>
 </sst>
 </file>
@@ -62749,7 +62866,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2DB8064-9FCF-4672-A5DD-AAA1AF5AE7B8}">
-  <dimension ref="A1:Z44"/>
+  <dimension ref="A1:Z83"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="50.90625" customWidth="1"/>
@@ -63254,7 +63371,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>583</v>
       </c>
@@ -63263,6 +63380,435 @@
       </c>
       <c r="C44" s="7">
         <v>46322</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="11" t="s">
+        <v>631</v>
+      </c>
+      <c r="B45" s="6" t="s">
+        <v>729</v>
+      </c>
+      <c r="C45" s="7">
+        <v>46323</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="11" t="s">
+        <v>632</v>
+      </c>
+      <c r="B46" s="6" t="s">
+        <v>730</v>
+      </c>
+      <c r="C46" s="7">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="11" t="s">
+        <v>633</v>
+      </c>
+      <c r="B47" s="6" t="s">
+        <v>731</v>
+      </c>
+      <c r="C47" s="7">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="11" t="s">
+        <v>634</v>
+      </c>
+      <c r="B48" s="6" t="s">
+        <v>732</v>
+      </c>
+      <c r="C48" s="7">
+        <v>46326</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="11" t="s">
+        <v>635</v>
+      </c>
+      <c r="B49" s="6" t="s">
+        <v>733</v>
+      </c>
+      <c r="C49" s="7">
+        <v>46327</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="11" t="s">
+        <v>636</v>
+      </c>
+      <c r="B50" s="6" t="s">
+        <v>734</v>
+      </c>
+      <c r="C50" s="7">
+        <v>46328</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="11" t="s">
+        <v>637</v>
+      </c>
+      <c r="B51" s="6" t="s">
+        <v>735</v>
+      </c>
+      <c r="C51" s="7">
+        <v>46329</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="11" t="s">
+        <v>638</v>
+      </c>
+      <c r="B52" s="6" t="s">
+        <v>736</v>
+      </c>
+      <c r="C52" s="7">
+        <v>46330</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="11" t="s">
+        <v>639</v>
+      </c>
+      <c r="B53" s="6" t="s">
+        <v>737</v>
+      </c>
+      <c r="C53" s="7">
+        <v>46331</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="11" t="s">
+        <v>640</v>
+      </c>
+      <c r="B54" s="6" t="s">
+        <v>738</v>
+      </c>
+      <c r="C54" s="7">
+        <v>46332</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="11" t="s">
+        <v>641</v>
+      </c>
+      <c r="B55" s="6" t="s">
+        <v>739</v>
+      </c>
+      <c r="C55" s="7">
+        <v>46333</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="11" t="s">
+        <v>642</v>
+      </c>
+      <c r="B56" s="6" t="s">
+        <v>740</v>
+      </c>
+      <c r="C56" s="7">
+        <v>46334</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A57" s="11" t="s">
+        <v>574</v>
+      </c>
+      <c r="B57" s="6" t="s">
+        <v>741</v>
+      </c>
+      <c r="C57" s="7">
+        <v>46335</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="11" t="s">
+        <v>643</v>
+      </c>
+      <c r="B58" s="6" t="s">
+        <v>742</v>
+      </c>
+      <c r="C58" s="7">
+        <v>46336</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="11" t="s">
+        <v>644</v>
+      </c>
+      <c r="B59" s="6" t="s">
+        <v>743</v>
+      </c>
+      <c r="C59" s="7">
+        <v>46337</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="11" t="s">
+        <v>645</v>
+      </c>
+      <c r="B60" s="6" t="s">
+        <v>744</v>
+      </c>
+      <c r="C60" s="7">
+        <v>46338</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="11" t="s">
+        <v>646</v>
+      </c>
+      <c r="B61" s="6" t="s">
+        <v>745</v>
+      </c>
+      <c r="C61" s="7">
+        <v>46339</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="11" t="s">
+        <v>647</v>
+      </c>
+      <c r="B62" s="6" t="s">
+        <v>746</v>
+      </c>
+      <c r="C62" s="7">
+        <v>46340</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A63" s="11" t="s">
+        <v>648</v>
+      </c>
+      <c r="B63" s="6" t="s">
+        <v>747</v>
+      </c>
+      <c r="C63" s="7">
+        <v>46341</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="11" t="s">
+        <v>648</v>
+      </c>
+      <c r="B64" s="6" t="s">
+        <v>748</v>
+      </c>
+      <c r="C64" s="7">
+        <v>46342</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A65" s="11" t="s">
+        <v>649</v>
+      </c>
+      <c r="B65" s="6" t="s">
+        <v>749</v>
+      </c>
+      <c r="C65" s="7">
+        <v>46343</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A66" s="11" t="s">
+        <v>650</v>
+      </c>
+      <c r="B66" s="6" t="s">
+        <v>750</v>
+      </c>
+      <c r="C66" s="7">
+        <v>46344</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A67" s="11" t="s">
+        <v>651</v>
+      </c>
+      <c r="B67" s="6" t="s">
+        <v>751</v>
+      </c>
+      <c r="C67" s="7">
+        <v>46345</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A68" s="11" t="s">
+        <v>652</v>
+      </c>
+      <c r="B68" s="6" t="s">
+        <v>752</v>
+      </c>
+      <c r="C68" s="7">
+        <v>46346</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A69" s="11" t="s">
+        <v>653</v>
+      </c>
+      <c r="B69" s="6" t="s">
+        <v>753</v>
+      </c>
+      <c r="C69" s="7">
+        <v>46347</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A70" s="11" t="s">
+        <v>654</v>
+      </c>
+      <c r="B70" s="6" t="s">
+        <v>754</v>
+      </c>
+      <c r="C70" s="7">
+        <v>46348</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A71" s="11" t="s">
+        <v>655</v>
+      </c>
+      <c r="B71" s="6" t="s">
+        <v>755</v>
+      </c>
+      <c r="C71" s="7">
+        <v>46349</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A72" s="11" t="s">
+        <v>656</v>
+      </c>
+      <c r="B72" s="6" t="s">
+        <v>756</v>
+      </c>
+      <c r="C72" s="7">
+        <v>46350</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A73" s="11" t="s">
+        <v>657</v>
+      </c>
+      <c r="B73" s="6" t="s">
+        <v>757</v>
+      </c>
+      <c r="C73" s="7">
+        <v>46351</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A74" s="11" t="s">
+        <v>658</v>
+      </c>
+      <c r="B74" s="6" t="s">
+        <v>758</v>
+      </c>
+      <c r="C74" s="7">
+        <v>46352</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A75" s="11" t="s">
+        <v>659</v>
+      </c>
+      <c r="B75" s="6" t="s">
+        <v>759</v>
+      </c>
+      <c r="C75" s="7">
+        <v>46353</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A76" s="11" t="s">
+        <v>660</v>
+      </c>
+      <c r="B76" s="6" t="s">
+        <v>760</v>
+      </c>
+      <c r="C76" s="7">
+        <v>46354</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A77" s="11" t="s">
+        <v>661</v>
+      </c>
+      <c r="B77" s="6" t="s">
+        <v>761</v>
+      </c>
+      <c r="C77" s="7">
+        <v>46355</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A78" s="11" t="s">
+        <v>662</v>
+      </c>
+      <c r="B78" s="6" t="s">
+        <v>762</v>
+      </c>
+      <c r="C78" s="7">
+        <v>46356</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A79" s="11" t="s">
+        <v>663</v>
+      </c>
+      <c r="B79" s="6" t="s">
+        <v>763</v>
+      </c>
+      <c r="C79" s="7">
+        <v>46357</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A80" s="11" t="s">
+        <v>664</v>
+      </c>
+      <c r="B80" s="6" t="s">
+        <v>764</v>
+      </c>
+      <c r="C80" s="7">
+        <v>46358</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A81" s="11" t="s">
+        <v>665</v>
+      </c>
+      <c r="B81" s="6" t="s">
+        <v>765</v>
+      </c>
+      <c r="C81" s="7">
+        <v>46359</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A82" s="11" t="s">
+        <v>666</v>
+      </c>
+      <c r="B82" s="6" t="s">
+        <v>766</v>
+      </c>
+      <c r="C82" s="7">
+        <v>46360</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A83" s="11" t="s">
+        <v>667</v>
+      </c>
+      <c r="B83" s="6" t="s">
+        <v>767</v>
+      </c>
+      <c r="C83" s="7">
+        <v>46361</v>
       </c>
     </row>
   </sheetData>
@@ -63270,6 +63816,45 @@
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1" display="https://www.youtube.com/watch?v=1Ilgi75Y6Ac&amp;t=9s" xr:uid="{BEFFE2FC-FF84-4042-B8EC-77144312CABC}"/>
     <hyperlink ref="A18" r:id="rId2" xr:uid="{266B1484-6826-4EF7-BFC0-E28E4199D83A}"/>
+    <hyperlink ref="A45" r:id="rId3" display="https://www.youtube.com/watch?v=Q24FZ2FRwGQ&amp;t=2s" xr:uid="{132FBFEE-56E3-4393-A4C6-D75016DECC29}"/>
+    <hyperlink ref="A46" r:id="rId4" xr:uid="{F50F6529-F0E8-4C70-A13D-64367A3A8066}"/>
+    <hyperlink ref="A47" r:id="rId5" display="https://www.youtube.com/watch?v=GTeBLRi-Hho&amp;t=1s" xr:uid="{08280529-3F60-4E29-9683-56CCE4D785D9}"/>
+    <hyperlink ref="A48" r:id="rId6" display="https://www.youtube.com/watch?v=AW19y7ztyKs&amp;t=1361s" xr:uid="{2F24D67A-527A-42EB-8910-2D49F1E87267}"/>
+    <hyperlink ref="A49" r:id="rId7" display="https://www.youtube.com/watch?v=nbGi3a_tyi0&amp;t=2s" xr:uid="{BA98A2AA-F4DC-4721-825C-4EFFB99F8B60}"/>
+    <hyperlink ref="A50" r:id="rId8" display="https://www.youtube.com/watch?v=QqTdOn-fxO4&amp;t=18s" xr:uid="{6EC6C4FD-8A9E-4F63-9D8C-F3335BE857A1}"/>
+    <hyperlink ref="A51" r:id="rId9" display="https://www.youtube.com/watch?v=z2dGDx3u5p0&amp;t=232s" xr:uid="{094927C5-447D-484A-BF4E-69DA11389CD0}"/>
+    <hyperlink ref="A52" r:id="rId10" display="https://www.youtube.com/watch?v=rPfM-T7cae8&amp;t=1s" xr:uid="{AEFCAA98-2FCE-4780-AA44-19FDEEFDE769}"/>
+    <hyperlink ref="A53" r:id="rId11" xr:uid="{5AE56921-6AAA-4AFA-B693-CDBFB6B4D107}"/>
+    <hyperlink ref="A54" r:id="rId12" display="https://www.youtube.com/watch?v=HLgoQEBcm6o&amp;t=125s" xr:uid="{37B80CBE-A48B-4672-B873-4A5D3383646C}"/>
+    <hyperlink ref="A55" r:id="rId13" display="https://www.youtube.com/watch?v=ruWNJ2f_KJs&amp;t=16s" xr:uid="{9942A07B-20B4-4CF9-A895-E7385BC32252}"/>
+    <hyperlink ref="A56" r:id="rId14" xr:uid="{AD7C63DF-8694-442F-A572-0E9A33676ADF}"/>
+    <hyperlink ref="A57" r:id="rId15" display="https://www.youtube.com/watch?v=ixeML2iYD3w&amp;t=3s" xr:uid="{BE8D5C45-9812-49AB-BBE6-0ADC09C426C7}"/>
+    <hyperlink ref="A58" r:id="rId16" xr:uid="{4BECC1C1-FB72-4D41-87FA-3EF76F012D22}"/>
+    <hyperlink ref="A59" r:id="rId17" display="https://www.youtube.com/watch?v=Lxwh9fSrLfo&amp;t=4s" xr:uid="{328B722C-0890-4DDE-8923-7A4B693829A6}"/>
+    <hyperlink ref="A60" r:id="rId18" xr:uid="{F6A13145-8D1C-46AA-9704-75C787042891}"/>
+    <hyperlink ref="A61" r:id="rId19" display="https://www.youtube.com/watch?v=Yjc7P_-Yuhg&amp;t=42s" xr:uid="{8CDE1602-3610-48CC-A2D0-8FCB57A22C4E}"/>
+    <hyperlink ref="A62" r:id="rId20" display="https://www.youtube.com/watch?v=Mv14PuzubPs&amp;t=2s" xr:uid="{F7F537A8-25FC-40AF-A10F-7D99E2120F20}"/>
+    <hyperlink ref="A63" r:id="rId21" display="https://www.youtube.com/watch?v=vVvHXSohHwA&amp;t=4s" xr:uid="{6D51514D-3752-4AF6-8619-09747580DFBD}"/>
+    <hyperlink ref="A64" r:id="rId22" display="https://www.youtube.com/watch?v=vVvHXSohHwA&amp;t=4s" xr:uid="{72878EB1-2699-450D-80A7-0F9C56FD1062}"/>
+    <hyperlink ref="A65" r:id="rId23" xr:uid="{3DD03F44-C4FC-4920-9CD4-EDFA9F623382}"/>
+    <hyperlink ref="A66" r:id="rId24" display="https://www.youtube.com/watch?v=TLaRnmjmabE&amp;t=2s" xr:uid="{82A29091-339B-49F2-AFB8-B501A153A69D}"/>
+    <hyperlink ref="A67" r:id="rId25" display="https://www.youtube.com/watch?v=8LGfGpiD-Mk&amp;t=11s" xr:uid="{2E223C6A-DDD3-49AC-8FF7-27C3CC856A44}"/>
+    <hyperlink ref="A68" r:id="rId26" display="https://www.youtube.com/watch?v=NrBla1RTvTE&amp;t=29s" xr:uid="{2B543A47-D491-44D9-ABCE-633213094941}"/>
+    <hyperlink ref="A69" r:id="rId27" xr:uid="{89AD0F73-85FA-483A-A254-5737A41B9834}"/>
+    <hyperlink ref="A70" r:id="rId28" xr:uid="{CD96F33B-8959-4F6A-B4D0-CFE7EA0265D3}"/>
+    <hyperlink ref="A71" r:id="rId29" xr:uid="{9C13BEFC-47F7-4727-9E09-034B59803FF2}"/>
+    <hyperlink ref="A72" r:id="rId30" xr:uid="{73ABE910-D2EF-4033-BE0E-73E900B50D1C}"/>
+    <hyperlink ref="A73" r:id="rId31" display="https://www.youtube.com/watch?v=Ai0jdNcEMHw&amp;t=5s" xr:uid="{F61408A1-CF32-473A-986E-2EF71CFAD396}"/>
+    <hyperlink ref="A74" r:id="rId32" xr:uid="{1577ACF6-79F3-4FE5-AEC5-983819FC0874}"/>
+    <hyperlink ref="A75" r:id="rId33" xr:uid="{2DA5147E-788D-4874-8CA4-AC1B4B921E94}"/>
+    <hyperlink ref="A76" r:id="rId34" xr:uid="{4FA474A0-92B8-4B33-A55E-90A47293767B}"/>
+    <hyperlink ref="A77" r:id="rId35" xr:uid="{6210D426-BED9-428D-9F42-25BB4934730B}"/>
+    <hyperlink ref="A78" r:id="rId36" xr:uid="{251C0452-33EC-42A1-BB0E-A4B0C5C69342}"/>
+    <hyperlink ref="A79" r:id="rId37" xr:uid="{9733D073-4C64-4755-9FF6-B7A256F84059}"/>
+    <hyperlink ref="A80" r:id="rId38" xr:uid="{631AB2C7-7C71-4BDB-84CE-4A4C255F65D4}"/>
+    <hyperlink ref="A81" r:id="rId39" xr:uid="{E0B9D2B7-76E4-40A7-975E-3B5174084D37}"/>
+    <hyperlink ref="A82" r:id="rId40" xr:uid="{61DE7A49-0711-4D44-8D25-E10CE16D756B}"/>
+    <hyperlink ref="A83" r:id="rId41" xr:uid="{7578719D-B46E-483D-8A0B-E16E12DBA4EC}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>